<commit_message>
Count September event ads at actual spend, separate from normal budget
SW2026 is recorded at the 48,422 yen actually spent instead of the 90,909 yen
reserve. September normal operations stay at 650,000 yen (normal_budget_ex_tax);
the unused reserve returns to the Oct-Apr allocation in the annual plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFkMa7pBd48FUqtUrcDcW8
</commit_message>
<xml_diff>
--- a/reports/売上目標_再設定_2026-09.xlsx
+++ b/reports/売上目標_再設定_2026-09.xlsx
@@ -814,10 +814,10 @@
         <v>1</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>740909</v>
+        <v>698422</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>100000</v>
+        <v>48422</v>
       </c>
       <c r="G22" s="11" t="n">
         <v>0.7</v>
@@ -844,7 +844,7 @@
         <v>1.1</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>1045713</v>
+        <v>1052086</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
@@ -869,7 +869,7 @@
         <v>1</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>1080570</v>
+        <v>1087156</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
         <v>1</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>1285141</v>
+        <v>1292364</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>100000</v>
@@ -919,7 +919,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>975999</v>
+        <v>981947</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>0</v>
@@ -944,7 +944,7 @@
         <v>0.75</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>1365427</v>
+        <v>1372225</v>
       </c>
       <c r="F27" s="6" t="n">
         <v>250000</v>
@@ -969,7 +969,7 @@
         <v>1</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>851713</v>
+        <v>856599</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>50000</v>
@@ -994,7 +994,7 @@
         <v>0.9</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>766856</v>
+        <v>771530</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>0</v>

</xml_diff>